<commit_message>
fix: harden v3.1.0 recovery and audit contracts
</commit_message>
<xml_diff>
--- a/assets/中台测试付款全量信息表.xlsx
+++ b/assets/中台测试付款全量信息表.xlsx
@@ -519,8 +519,8 @@
   <dimension ref="A1:AF1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="2" width="14" customWidth="1"/>
-    <col min="3" max="4" width="14" style="1" customWidth="1"/>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="4" width="14" style="1" customWidth="1"/>
     <col min="5" max="14" width="14" customWidth="1"/>
     <col min="15" max="15" width="14" style="1" customWidth="1"/>
     <col min="16" max="18" width="14" customWidth="1"/>
@@ -539,7 +539,7 @@
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="3" t="s">

</xml_diff>